<commit_message>
Apply user card tweaks from the balancing sheet
- Deeper Cold: chill slow 0.08 -> 0.2, promoted common -> rare
- Goblin War-Hymn: no longer unique (copies stack to 4x in the window)
- New: Skywatch 2 (+50% vs flying, rare, unique) — id de-duplicated
  from the sheet's pr_skywatch to pr_skywatch2

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wildguard-cards.xlsx
+++ b/wildguard-cards.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX54"/>
+  <dimension ref="A1:AX55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Chill slows +8% more</t>
+          <t>Chill slows +20% more</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -1221,7 +1221,7 @@
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>common</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="H7" s="6" t="n"/>
@@ -1233,7 +1233,7 @@
       <c r="N7" s="7" t="n"/>
       <c r="O7" s="7" t="n"/>
       <c r="P7" s="7" t="n">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="Q7" s="7" t="n"/>
       <c r="R7" s="7" t="n"/>
@@ -4374,11 +4374,7 @@
           <t>uncommon</t>
         </is>
       </c>
-      <c r="H46" s="6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+      <c r="H46" s="6" t="n"/>
       <c r="I46" s="7" t="n"/>
       <c r="J46" s="7" t="n"/>
       <c r="K46" s="7" t="n"/>
@@ -5108,21 +5104,103 @@
         <v>1.25</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>pr_skywatch2</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>Skywatch 2</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>ALL towers deal +50% damage to FLYING enemies</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>🦅</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n"/>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="n"/>
+      <c r="J55" s="7" t="n"/>
+      <c r="K55" s="7" t="n"/>
+      <c r="L55" s="7" t="n"/>
+      <c r="M55" s="7" t="n"/>
+      <c r="N55" s="7" t="n"/>
+      <c r="O55" s="7" t="n"/>
+      <c r="P55" s="7" t="n"/>
+      <c r="Q55" s="7" t="n"/>
+      <c r="R55" s="7" t="n"/>
+      <c r="S55" s="7" t="n"/>
+      <c r="T55" s="7" t="n"/>
+      <c r="U55" s="7" t="n"/>
+      <c r="V55" s="7" t="n"/>
+      <c r="W55" s="7" t="n"/>
+      <c r="X55" s="7" t="n"/>
+      <c r="Y55" s="7" t="n"/>
+      <c r="Z55" s="7" t="n"/>
+      <c r="AA55" s="7" t="n"/>
+      <c r="AB55" s="7" t="n"/>
+      <c r="AC55" s="7" t="n"/>
+      <c r="AD55" s="7" t="n"/>
+      <c r="AE55" s="7" t="n"/>
+      <c r="AF55" s="7" t="n"/>
+      <c r="AG55" s="7" t="n"/>
+      <c r="AH55" s="7" t="n"/>
+      <c r="AI55" s="7" t="n"/>
+      <c r="AJ55" s="7" t="n"/>
+      <c r="AK55" s="7" t="n"/>
+      <c r="AL55" s="7" t="n"/>
+      <c r="AM55" s="7" t="n"/>
+      <c r="AN55" s="7" t="n"/>
+      <c r="AO55" s="7" t="n"/>
+      <c r="AP55" s="7" t="n"/>
+      <c r="AQ55" s="7" t="n"/>
+      <c r="AR55" s="7" t="n"/>
+      <c r="AS55" s="7" t="n"/>
+      <c r="AT55" s="7" t="n"/>
+      <c r="AU55" s="7" t="n"/>
+      <c r="AV55" s="7" t="n"/>
+      <c r="AW55" s="7" t="n"/>
+      <c r="AX55" s="7" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="E2:E113" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E114" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"fire,ice,lightning,water,wind,physical,void,all"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F113" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F114" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"wizard,goblin,archer,tree,void"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G113" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G114" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"common,uncommon,rare"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H113" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H114" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"TRUE"</formula1>
     </dataValidation>
-    <dataValidation sqref="AR2:AR113" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="AR2:AR114" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"rattled,wet,chill,frozen,burn,entangled"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5311,7 +5389,7 @@
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>Current pool: 53 cards. Water-mage cards removed; 5 new Void cards (void_dmg1, void_rate1, void_range1, void_splash1, void_dmg2).</t>
+          <t>Current pool: 54 cards. Water-mage cards removed; 5 new Void cards (void_dmg1, void_rate1, void_range1, void_splash1, void_dmg2).</t>
         </is>
       </c>
     </row>

</xml_diff>